<commit_message>
haven't done this in a while
</commit_message>
<xml_diff>
--- a/tentative lab schedule.xlsx
+++ b/tentative lab schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac6229071bdafc06/UVI/F26_MES503/MES503Lab/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{E744A197-76D0-4E27-9ED7-A75E497808E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EF88C97-D1A2-42D8-A60D-75B40138ABDC}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{E744A197-76D0-4E27-9ED7-A75E497808E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{222F7419-74F3-4E5B-9FB2-D807464D7C84}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{5D9DF16E-F8C4-45DA-8F92-13F2A9E88223}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{5D9DF16E-F8C4-45DA-8F92-13F2A9E88223}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>MES 503 Lab Tentative Schedule</t>
   </si>
@@ -83,9 +83,6 @@
     <t>filter()/select()/arrange()</t>
   </si>
   <si>
-    <t>group_by()/summarize()</t>
-  </si>
-  <si>
     <t>joins()</t>
   </si>
   <si>
@@ -110,19 +107,31 @@
     <t>for loops</t>
   </si>
   <si>
+    <t>NA (Labor Day)</t>
+  </si>
+  <si>
+    <t>Multiple Regression</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>group_by()/summarize()/mutate()</t>
+  </si>
+  <si>
+    <t>functions- Spring MES 504</t>
+  </si>
+  <si>
     <t>functions</t>
   </si>
   <si>
-    <t>NA (Labor Day)</t>
-  </si>
-  <si>
-    <t>Multiple Regression</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>intro to data wrangling</t>
+    <t>dates/times</t>
+  </si>
+  <si>
+    <t>functions/dates/times review</t>
+  </si>
+  <si>
+    <t>Integrate everything we have done - coding escape room? Haunted House themed</t>
   </si>
 </sst>
 </file>
@@ -184,10 +193,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -513,6 +518,7 @@
     <col min="2" max="2" width="23.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.08984375" customWidth="1"/>
+    <col min="7" max="7" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -534,7 +540,7 @@
         <v>4</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -548,7 +554,7 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
@@ -559,10 +565,10 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
@@ -573,7 +579,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -581,10 +587,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -598,7 +604,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -609,7 +615,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D8">
         <v>2</v>
@@ -623,7 +629,7 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -634,7 +640,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -642,10 +648,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -659,7 +665,7 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
@@ -670,10 +676,13 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D13">
         <v>4</v>
+      </c>
+      <c r="G13" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
@@ -681,10 +690,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>